<commit_message>
Upload October_26_Utilities_Tracking.xlsx via dashboard admin
</commit_message>
<xml_diff>
--- a/data/raw/October_26_Utilities_Tracking.xlsx
+++ b/data/raw/October_26_Utilities_Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\UTILITIES\Tracking\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585977AC-6ABF-4180-8504-7477A909231A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFB328F-B997-47AD-AF4A-C1C938BEF167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="579" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -235,7 +235,7 @@
           <t xml:space="preserve">Tank A 0 kgs 
 Tank B 0 kgs
 Tank C 16300 Kgs
-mobile approx 19600 Kgs
+mobile approx 18900Kgs
 0 kgs after adjustment for MT mobile weight
 </t>
         </r>
@@ -253,7 +253,169 @@
           <t xml:space="preserve">Tank A 0 kgs 
 Tank B 0 kgs
 Tank C 25700 Kgs
-mobile approx 8600 Kgs
+mobile approx 7900 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D74" authorId="2" shapeId="0" xr:uid="{A9D615D0-28C9-4C13-9020-A7C276975F57}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 6700 kgs calculated
+Tank C 25700 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F74" authorId="2" shapeId="0" xr:uid="{B1148AEC-E522-4F72-A286-908A2BFB66B0}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 6700 kgs calculated
+Tank C 25700 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G74" authorId="2" shapeId="0" xr:uid="{72907FFC-D535-40B6-B65A-2A5AE920A761}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 5100 kgs calculated
+Tank C 25700 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H74" authorId="2" shapeId="0" xr:uid="{A350E13C-FC63-4A46-AEC7-D15BEAB66A89}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 3600 kgs calculated
+Tank C 25700 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I74" authorId="2" shapeId="0" xr:uid="{70143B87-12C5-483A-9CF2-B1AD2D0FFF73}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 2200 kgs calculated
+Tank C 25700 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J74" authorId="2" shapeId="0" xr:uid="{F10121C0-B811-45B6-8088-211B562FC585}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 0 kgs calculated
+Tank C 24900 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K74" authorId="2" shapeId="0" xr:uid="{7E734BED-4455-464B-B3BC-84E273292C6E}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 0 kgs 
+Tank C 23200 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L74" authorId="2" shapeId="0" xr:uid="{EDC26567-6215-4B13-89B4-8CB9A2D8B046}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 0 kgs
+Tank C 22400 Kgs
+mobile approx 0 Kgs
+0 kgs after adjustment for MT mobile weight
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M74" authorId="2" shapeId="0" xr:uid="{88951BC3-57B8-4D8F-9300-706887E45023}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tank A 0 kgs 
+Tank B 0 kgs
+Tank C 22400 Kgs
+mobile approx 20800 Kgs
 0 kgs after adjustment for MT mobile weight
 </t>
         </r>
@@ -311,7 +473,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="314">
   <si>
     <t>UTILITY ANALYSIS</t>
   </si>
@@ -2896,6 +3058,9 @@
   </si>
   <si>
     <t>ST/CB</t>
+  </si>
+  <si>
+    <t>GU</t>
   </si>
 </sst>
 </file>
@@ -5991,7 +6156,7 @@
     <xf numFmtId="9" fontId="49" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="172" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1024">
+  <cellXfs count="1027">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -8423,6 +8588,12 @@
     <xf numFmtId="0" fontId="104" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="75" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="75" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="77" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -8809,6 +8980,9 @@
     </xf>
     <xf numFmtId="167" fontId="69" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="95" fillId="31" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -8819,477 +8993,7 @@
     <cellStyle name="Normal_February04" xfId="3" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Percent" xfId="4" builtinId="5"/>
   </cellStyles>
-  <dxfs count="167">
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="120">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -12594,53 +12298,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" ht="18" x14ac:dyDescent="0.2">
-      <c r="B1" s="899" t="s">
+      <c r="B1" s="901" t="s">
         <v>209</v>
       </c>
-      <c r="C1" s="899"/>
-      <c r="D1" s="899"/>
-      <c r="E1" s="899"/>
-      <c r="F1" s="899"/>
-      <c r="G1" s="899"/>
-      <c r="H1" s="899"/>
-      <c r="I1" s="899"/>
-      <c r="J1" s="899"/>
-      <c r="K1" s="899"/>
-      <c r="L1" s="899"/>
-      <c r="M1" s="899"/>
+      <c r="C1" s="901"/>
+      <c r="D1" s="901"/>
+      <c r="E1" s="901"/>
+      <c r="F1" s="901"/>
+      <c r="G1" s="901"/>
+      <c r="H1" s="901"/>
+      <c r="I1" s="901"/>
+      <c r="J1" s="901"/>
+      <c r="K1" s="901"/>
+      <c r="L1" s="901"/>
+      <c r="M1" s="901"/>
       <c r="N1" s="363"/>
-      <c r="O1" s="900" t="str">
+      <c r="O1" s="902" t="str">
         <f>B1</f>
         <v>ENTRIES FOR DAILY CONS. MONITOR</v>
       </c>
-      <c r="P1" s="900"/>
-      <c r="Q1" s="900"/>
-      <c r="R1" s="900"/>
-      <c r="S1" s="900"/>
-      <c r="T1" s="900"/>
-      <c r="U1" s="900"/>
-      <c r="V1" s="900"/>
-      <c r="W1" s="900"/>
-      <c r="X1" s="900"/>
-      <c r="Y1" s="900"/>
-      <c r="Z1" s="900"/>
-      <c r="AA1" s="900"/>
-      <c r="AB1" s="900"/>
+      <c r="P1" s="902"/>
+      <c r="Q1" s="902"/>
+      <c r="R1" s="902"/>
+      <c r="S1" s="902"/>
+      <c r="T1" s="902"/>
+      <c r="U1" s="902"/>
+      <c r="V1" s="902"/>
+      <c r="W1" s="902"/>
+      <c r="X1" s="902"/>
+      <c r="Y1" s="902"/>
+      <c r="Z1" s="902"/>
+      <c r="AA1" s="902"/>
+      <c r="AB1" s="902"/>
     </row>
     <row r="2" spans="1:44" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C2" s="810"/>
       <c r="F2" s="364"/>
       <c r="G2" s="365"/>
-      <c r="O2" s="908" t="s">
+      <c r="O2" s="910" t="s">
         <v>231</v>
       </c>
-      <c r="P2" s="908"/>
-      <c r="Q2" s="908"/>
-      <c r="R2" s="908"/>
-      <c r="S2" s="908"/>
-      <c r="T2" s="908"/>
-      <c r="U2" s="908"/>
-      <c r="V2" s="908"/>
+      <c r="P2" s="910"/>
+      <c r="Q2" s="910"/>
+      <c r="R2" s="910"/>
+      <c r="S2" s="910"/>
+      <c r="T2" s="910"/>
+      <c r="U2" s="910"/>
+      <c r="V2" s="910"/>
     </row>
     <row r="3" spans="1:44" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="366"/>
@@ -12658,50 +12362,50 @@
         <v>22</v>
       </c>
       <c r="K3" s="369"/>
-      <c r="L3" s="913" t="s">
+      <c r="L3" s="915" t="s">
         <v>53</v>
       </c>
-      <c r="M3" s="914"/>
-      <c r="N3" s="915"/>
-      <c r="O3" s="901" t="s">
+      <c r="M3" s="916"/>
+      <c r="N3" s="917"/>
+      <c r="O3" s="903" t="s">
         <v>3</v>
       </c>
-      <c r="P3" s="901"/>
-      <c r="Q3" s="901"/>
-      <c r="R3" s="901"/>
-      <c r="S3" s="901"/>
-      <c r="T3" s="901"/>
-      <c r="U3" s="901"/>
-      <c r="V3" s="901"/>
-      <c r="W3" s="901"/>
-      <c r="X3" s="901"/>
-      <c r="Y3" s="901"/>
-      <c r="Z3" s="901"/>
-      <c r="AA3" s="901"/>
-      <c r="AB3" s="901"/>
-      <c r="AC3" s="901"/>
+      <c r="P3" s="903"/>
+      <c r="Q3" s="903"/>
+      <c r="R3" s="903"/>
+      <c r="S3" s="903"/>
+      <c r="T3" s="903"/>
+      <c r="U3" s="903"/>
+      <c r="V3" s="903"/>
+      <c r="W3" s="903"/>
+      <c r="X3" s="903"/>
+      <c r="Y3" s="903"/>
+      <c r="Z3" s="903"/>
+      <c r="AA3" s="903"/>
+      <c r="AB3" s="903"/>
+      <c r="AC3" s="903"/>
       <c r="AD3" s="372"/>
       <c r="AE3" s="373"/>
       <c r="AF3" s="372"/>
-      <c r="AG3" s="921" t="s">
+      <c r="AG3" s="923" t="s">
         <v>206</v>
       </c>
-      <c r="AH3" s="919" t="s">
+      <c r="AH3" s="921" t="s">
         <v>204</v>
       </c>
-      <c r="AI3" s="919" t="s">
+      <c r="AI3" s="921" t="s">
         <v>205</v>
       </c>
-      <c r="AJ3" s="922" t="s">
+      <c r="AJ3" s="924" t="s">
         <v>233</v>
       </c>
       <c r="AK3" s="416"/>
-      <c r="AL3" s="923" t="s">
+      <c r="AL3" s="925" t="s">
         <v>178</v>
       </c>
-      <c r="AM3" s="923"/>
-      <c r="AN3" s="923"/>
-      <c r="AO3" s="923"/>
+      <c r="AM3" s="925"/>
+      <c r="AN3" s="925"/>
+      <c r="AO3" s="925"/>
     </row>
     <row r="4" spans="1:44" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="374"/>
@@ -12735,40 +12439,40 @@
       <c r="K4" s="372" t="s">
         <v>31</v>
       </c>
-      <c r="L4" s="909" t="s">
+      <c r="L4" s="911" t="s">
         <v>289</v>
       </c>
       <c r="M4" s="376" t="s">
         <v>260</v>
       </c>
-      <c r="N4" s="916" t="s">
+      <c r="N4" s="918" t="s">
         <v>167</v>
       </c>
-      <c r="O4" s="897" t="s">
+      <c r="O4" s="899" t="s">
         <v>100</v>
       </c>
-      <c r="P4" s="897" t="s">
+      <c r="P4" s="899" t="s">
         <v>101</v>
       </c>
-      <c r="Q4" s="897" t="s">
+      <c r="Q4" s="899" t="s">
         <v>160</v>
       </c>
-      <c r="R4" s="897" t="s">
+      <c r="R4" s="899" t="s">
         <v>171</v>
       </c>
-      <c r="S4" s="897" t="s">
+      <c r="S4" s="899" t="s">
         <v>102</v>
       </c>
-      <c r="T4" s="897" t="s">
+      <c r="T4" s="899" t="s">
         <v>172</v>
       </c>
-      <c r="U4" s="897" t="s">
+      <c r="U4" s="899" t="s">
         <v>103</v>
       </c>
-      <c r="V4" s="906" t="s">
+      <c r="V4" s="908" t="s">
         <v>236</v>
       </c>
-      <c r="W4" s="897" t="s">
+      <c r="W4" s="899" t="s">
         <v>177</v>
       </c>
       <c r="X4" s="372" t="s">
@@ -12780,28 +12484,28 @@
       <c r="Z4" s="372" t="s">
         <v>98</v>
       </c>
-      <c r="AA4" s="901" t="s">
+      <c r="AA4" s="903" t="s">
         <v>68</v>
       </c>
-      <c r="AB4" s="903" t="s">
+      <c r="AB4" s="905" t="s">
         <v>69</v>
       </c>
-      <c r="AC4" s="907" t="s">
+      <c r="AC4" s="909" t="s">
         <v>151</v>
       </c>
-      <c r="AD4" s="897" t="s">
+      <c r="AD4" s="899" t="s">
         <v>154</v>
       </c>
-      <c r="AE4" s="897" t="s">
+      <c r="AE4" s="899" t="s">
         <v>155</v>
       </c>
-      <c r="AF4" s="897" t="s">
+      <c r="AF4" s="899" t="s">
         <v>159</v>
       </c>
-      <c r="AG4" s="921"/>
-      <c r="AH4" s="920"/>
-      <c r="AI4" s="920"/>
-      <c r="AJ4" s="922"/>
+      <c r="AG4" s="923"/>
+      <c r="AH4" s="922"/>
+      <c r="AI4" s="922"/>
+      <c r="AJ4" s="924"/>
       <c r="AK4" s="416"/>
       <c r="AL4" s="378" t="s">
         <v>276</v>
@@ -12850,20 +12554,20 @@
       <c r="K5" s="465" t="s">
         <v>36</v>
       </c>
-      <c r="L5" s="910"/>
+      <c r="L5" s="912"/>
       <c r="M5" s="466" t="s">
         <v>261</v>
       </c>
-      <c r="N5" s="917"/>
-      <c r="O5" s="905"/>
-      <c r="P5" s="897"/>
-      <c r="Q5" s="897"/>
-      <c r="R5" s="897"/>
-      <c r="S5" s="905"/>
-      <c r="T5" s="905"/>
-      <c r="U5" s="905"/>
-      <c r="V5" s="906"/>
-      <c r="W5" s="918"/>
+      <c r="N5" s="919"/>
+      <c r="O5" s="907"/>
+      <c r="P5" s="899"/>
+      <c r="Q5" s="899"/>
+      <c r="R5" s="899"/>
+      <c r="S5" s="907"/>
+      <c r="T5" s="907"/>
+      <c r="U5" s="907"/>
+      <c r="V5" s="908"/>
+      <c r="W5" s="920"/>
       <c r="X5" s="372" t="s">
         <v>104</v>
       </c>
@@ -12873,16 +12577,16 @@
       <c r="Z5" s="372" t="s">
         <v>104</v>
       </c>
-      <c r="AA5" s="902"/>
-      <c r="AB5" s="904"/>
-      <c r="AC5" s="907"/>
-      <c r="AD5" s="897"/>
-      <c r="AE5" s="897"/>
-      <c r="AF5" s="898"/>
-      <c r="AG5" s="921"/>
-      <c r="AH5" s="920"/>
-      <c r="AI5" s="920"/>
-      <c r="AJ5" s="922"/>
+      <c r="AA5" s="904"/>
+      <c r="AB5" s="906"/>
+      <c r="AC5" s="909"/>
+      <c r="AD5" s="899"/>
+      <c r="AE5" s="899"/>
+      <c r="AF5" s="900"/>
+      <c r="AG5" s="923"/>
+      <c r="AH5" s="922"/>
+      <c r="AI5" s="922"/>
+      <c r="AJ5" s="924"/>
       <c r="AK5" s="416"/>
       <c r="AL5" s="378" t="s">
         <v>263</v>
@@ -14899,8 +14603,8 @@
     <row r="38" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B38" s="190"/>
       <c r="G38" s="190"/>
-      <c r="I38" s="911"/>
-      <c r="J38" s="911"/>
+      <c r="I38" s="913"/>
+      <c r="J38" s="913"/>
       <c r="R38" s="190"/>
       <c r="S38" s="190"/>
       <c r="T38" s="190"/>
@@ -14908,8 +14612,8 @@
       <c r="V38" s="190"/>
       <c r="W38" s="190"/>
       <c r="Z38" s="190"/>
-      <c r="AA38" s="912"/>
-      <c r="AB38" s="912"/>
+      <c r="AA38" s="914"/>
+      <c r="AB38" s="914"/>
       <c r="AC38" s="190"/>
       <c r="AD38" s="190"/>
       <c r="AI38" s="380"/>
@@ -16606,404 +16310,289 @@
     <mergeCell ref="L4:L5"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
-  <conditionalFormatting sqref="B18:B35">
-    <cfRule type="expression" dxfId="165" priority="75">
-      <formula>B18&lt;B17</formula>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="expression" dxfId="119" priority="14">
+      <formula>B6&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:B35">
+    <cfRule type="expression" dxfId="118" priority="28">
+      <formula>B7&lt;B6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11:B17">
+    <cfRule type="expression" dxfId="117" priority="45">
+      <formula>B11&lt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C35 E35:E37">
-    <cfRule type="expression" dxfId="163" priority="380">
+    <cfRule type="expression" dxfId="116" priority="380">
       <formula>C35&lt;C34</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C6:D6">
+    <cfRule type="expression" dxfId="115" priority="16">
+      <formula>C6&lt;C5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7:D7 H7:J7 R7 T7 W7 AB7">
+    <cfRule type="expression" dxfId="114" priority="32">
+      <formula>C7&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C8:D14">
+    <cfRule type="expression" dxfId="113" priority="36">
+      <formula>C8&lt;C7</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C36:D37">
-    <cfRule type="expression" dxfId="159" priority="1433">
+    <cfRule type="expression" dxfId="112" priority="1433">
       <formula>C36&lt;C35</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D35 B36:B37">
-    <cfRule type="expression" dxfId="158" priority="1420">
+    <cfRule type="expression" dxfId="111" priority="1420">
       <formula>B35&lt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F18:F37">
-    <cfRule type="expression" dxfId="156" priority="51">
-      <formula>F18&lt;#REF!</formula>
+  <conditionalFormatting sqref="E6:E14">
+    <cfRule type="expression" dxfId="110" priority="5">
+      <formula>E6&lt;E5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G18:G37">
-    <cfRule type="expression" dxfId="155" priority="49">
-      <formula>G18&lt;G17</formula>
+  <conditionalFormatting sqref="F6:F37">
+    <cfRule type="expression" dxfId="109" priority="4">
+      <formula>F6&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:G37">
+    <cfRule type="expression" dxfId="108" priority="2">
+      <formula>G6&lt;G5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G36:J37 L36:O37">
-    <cfRule type="expression" dxfId="154" priority="1267">
+    <cfRule type="expression" dxfId="107" priority="1267">
       <formula>G36&lt;G35</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G6:O6">
+    <cfRule type="expression" dxfId="106" priority="6">
+      <formula>G6&lt;G5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H19:I34">
-    <cfRule type="expression" dxfId="152" priority="381">
+    <cfRule type="expression" dxfId="105" priority="381">
       <formula>H19&lt;H18</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H35:I35 R35 T35 W35 AB35 AE35:AI35 P36:P37 S36:S37 X36:Y37">
-    <cfRule type="expression" dxfId="151" priority="1419">
+    <cfRule type="expression" dxfId="104" priority="1419">
       <formula>H35&lt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H18:J18">
-    <cfRule type="expression" dxfId="150" priority="84">
-      <formula>H18&lt;H17</formula>
+  <conditionalFormatting sqref="H8:J18">
+    <cfRule type="expression" dxfId="103" priority="37">
+      <formula>H8&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J19:J35">
-    <cfRule type="expression" dxfId="149" priority="382">
+    <cfRule type="expression" dxfId="102" priority="382">
       <formula>J19&lt;J18</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K18:L21">
-    <cfRule type="expression" dxfId="148" priority="87">
-      <formula>K18&lt;K17</formula>
+  <conditionalFormatting sqref="K11:L21">
+    <cfRule type="expression" dxfId="101" priority="40">
+      <formula>K11&lt;K10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K22:M22">
-    <cfRule type="expression" dxfId="147" priority="383">
+    <cfRule type="expression" dxfId="100" priority="383">
       <formula>K22&lt;K21</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K7:O10">
+    <cfRule type="expression" dxfId="99" priority="23">
+      <formula>K7&lt;K6</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K23:Z23 K24:K37">
-    <cfRule type="expression" dxfId="145" priority="384">
+    <cfRule type="expression" dxfId="98" priority="384">
       <formula>K23&lt;K22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L24:Z27 L28:AC28">
-    <cfRule type="expression" dxfId="144" priority="386">
+    <cfRule type="expression" dxfId="97" priority="386">
       <formula>L24&lt;L23</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="M11:M17">
+    <cfRule type="expression" dxfId="96" priority="42">
+      <formula>M11&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M18:M21">
-    <cfRule type="expression" dxfId="142" priority="379">
+    <cfRule type="expression" dxfId="95" priority="379">
       <formula>M18&lt;M17</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N18:T22">
-    <cfRule type="expression" dxfId="140" priority="91">
-      <formula>N18&lt;N17</formula>
+  <conditionalFormatting sqref="N11:O12">
+    <cfRule type="expression" dxfId="94" priority="41">
+      <formula>N11&lt;N10</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N13:T22">
+    <cfRule type="expression" dxfId="93" priority="44">
+      <formula>N13&lt;N12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P8:P12 V8:V12">
+    <cfRule type="expression" dxfId="92" priority="39">
+      <formula>P8&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P6:Q6 X6:Y6 S6:S10">
+    <cfRule type="expression" dxfId="91" priority="13">
+      <formula>P6&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P7:Q7">
+    <cfRule type="expression" dxfId="90" priority="30">
+      <formula>P7&lt;P6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q36">
-    <cfRule type="expression" dxfId="136" priority="1436">
+    <cfRule type="expression" dxfId="89" priority="1436">
       <formula>Q36&lt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q8:R10">
+    <cfRule type="expression" dxfId="88" priority="38">
+      <formula>Q8&lt;Q7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:T12">
+    <cfRule type="expression" dxfId="87" priority="43">
+      <formula>Q11&lt;Q10</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R6">
+    <cfRule type="expression" dxfId="86" priority="15">
+      <formula>R6&lt;R5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="R36">
-    <cfRule type="expression" dxfId="132" priority="1432">
+    <cfRule type="expression" dxfId="85" priority="1432">
       <formula>R36&lt;R35</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB18:AI27">
-    <cfRule type="expression" dxfId="131" priority="81">
-      <formula>AB18&lt;AB17</formula>
+  <conditionalFormatting sqref="T8:T10 AB8:AC10 AE8:AI10 AB11:AI27">
+    <cfRule type="expression" dxfId="84" priority="34">
+      <formula>T8&lt;T7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U18:U22">
-    <cfRule type="expression" dxfId="129" priority="56">
-      <formula>U18&lt;U17</formula>
+  <conditionalFormatting sqref="T6:W6 Z6 AB6">
+    <cfRule type="expression" dxfId="83" priority="12">
+      <formula>T6&lt;T5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18:E34">
-    <cfRule type="expression" dxfId="127" priority="94">
-      <formula>C18&lt;C17</formula>
+  <conditionalFormatting sqref="U6:U22">
+    <cfRule type="expression" dxfId="82" priority="9">
+      <formula>U6&lt;U5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V18:Z22">
-    <cfRule type="expression" dxfId="126" priority="93">
-      <formula>V18&lt;V17</formula>
+  <conditionalFormatting sqref="V7">
+    <cfRule type="expression" dxfId="81" priority="25">
+      <formula>V7&lt;V6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V13:X14 C15:E34">
+    <cfRule type="expression" dxfId="80" priority="47">
+      <formula>C13&lt;C12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V15:Z22">
+    <cfRule type="expression" dxfId="79" priority="46">
+      <formula>V15&lt;V14</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V29:AC29 AA30:AC30 Z30:Z31 V30:Y34 AA31:AB31 AC31:AC37 Z32:AB34 V35 X35:AA35">
-    <cfRule type="expression" dxfId="125" priority="390">
+    <cfRule type="expression" dxfId="78" priority="390">
       <formula>V29&lt;V28</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA18:AA37">
-    <cfRule type="expression" dxfId="121" priority="48">
-      <formula>AA18&lt;AA17</formula>
+  <conditionalFormatting sqref="W8:W12">
+    <cfRule type="expression" dxfId="77" priority="35">
+      <formula>W8&lt;W7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y7:Z14">
+    <cfRule type="expression" dxfId="76" priority="26">
+      <formula>Y7&lt;Y6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA6:AA12">
+    <cfRule type="expression" dxfId="75" priority="8">
+      <formula>AA6&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA6:AA37">
+    <cfRule type="expression" dxfId="74" priority="1">
+      <formula>AA6&lt;AA5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA28:AA37">
-    <cfRule type="expression" dxfId="120" priority="388">
+    <cfRule type="expression" dxfId="73" priority="388">
       <formula>AA28&lt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AC6:AC7">
+    <cfRule type="expression" dxfId="72" priority="10">
+      <formula>AC6&lt;AC5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AD28:AD37">
-    <cfRule type="expression" dxfId="118" priority="385">
+    <cfRule type="expression" dxfId="71" priority="385">
       <formula>AD28&lt;AD27</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AD6:AI6">
+    <cfRule type="expression" dxfId="70" priority="7">
+      <formula>AD6&lt;AD5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AI7 X7:X12 AD8:AD10">
+    <cfRule type="expression" dxfId="69" priority="27">
+      <formula>X7&lt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AE28:AI34 L29:T34 U29:U37 L35:Q35 S35">
-    <cfRule type="expression" dxfId="115" priority="389">
+    <cfRule type="expression" dxfId="68" priority="389">
       <formula>L28&lt;L27</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ18:AJ37">
-    <cfRule type="expression" dxfId="114" priority="50">
-      <formula>AJ18&lt;AJ17</formula>
+  <conditionalFormatting sqref="AJ6:AJ37">
+    <cfRule type="expression" dxfId="67" priority="3">
+      <formula>AJ6&lt;AJ5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK6:AK12">
-    <cfRule type="expression" dxfId="113" priority="1309">
+    <cfRule type="expression" dxfId="66" priority="1309">
       <formula>AK6&lt;AK5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK13:AL15">
-    <cfRule type="expression" dxfId="112" priority="1389">
+    <cfRule type="expression" dxfId="65" priority="1389">
       <formula>AK13&lt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL9:AL14 AL15:AN34 AK16:AK37 AK20:AN21 T36:W37 Z36:Z37 AB36:AB37 AE36:AI37 Q37:R37">
-    <cfRule type="expression" dxfId="111" priority="1326">
+    <cfRule type="expression" dxfId="64" priority="1326">
       <formula>Q9&lt;Q8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO9:AO34">
-    <cfRule type="expression" dxfId="110" priority="1334">
+    <cfRule type="expression" dxfId="63" priority="1334">
       <formula>AO9&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B7:B17">
-    <cfRule type="expression" dxfId="46" priority="28">
-      <formula>B7&lt;B6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11:B17">
-    <cfRule type="expression" dxfId="45" priority="45">
-      <formula>B11&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7:D7 H7:J7 R7 T7 W7 AB7">
-    <cfRule type="expression" dxfId="44" priority="32">
-      <formula>C7&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8:D14">
-    <cfRule type="expression" dxfId="43" priority="36">
-      <formula>C8&lt;C7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E14">
-    <cfRule type="expression" dxfId="42" priority="18">
-      <formula>E7&lt;E6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F17">
-    <cfRule type="expression" dxfId="41" priority="33">
-      <formula>F7&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G17">
-    <cfRule type="expression" dxfId="40" priority="29">
-      <formula>G7&lt;G6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H8:J17">
-    <cfRule type="expression" dxfId="39" priority="37">
-      <formula>H8&lt;H7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11:L17">
-    <cfRule type="expression" dxfId="38" priority="40">
-      <formula>K11&lt;K10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:O8 K9:N10 O9">
-    <cfRule type="expression" dxfId="37" priority="23">
-      <formula>K7&lt;K6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M11:M17">
-    <cfRule type="expression" dxfId="36" priority="42">
-      <formula>M11&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N11:O12 O10">
-    <cfRule type="expression" dxfId="35" priority="41">
-      <formula>N10&lt;N9</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N13:T17">
-    <cfRule type="expression" dxfId="34" priority="44">
-      <formula>N13&lt;N12</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S7:S10">
-    <cfRule type="expression" dxfId="33" priority="22">
-      <formula>S7&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P8:P12 V8:V12">
-    <cfRule type="expression" dxfId="32" priority="39">
-      <formula>P8&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P7:Q7">
-    <cfRule type="expression" dxfId="31" priority="30">
-      <formula>P7&lt;P6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q8:R8">
-    <cfRule type="expression" dxfId="30" priority="38">
-      <formula>Q8&lt;Q7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:T12 Q9:R10 T9:T10">
-    <cfRule type="expression" dxfId="29" priority="43">
-      <formula>Q9&lt;Q8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T8 AB8:AC10 AE8:AI10 AB11:AI17">
-    <cfRule type="expression" dxfId="28" priority="34">
-      <formula>T8&lt;T7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U17">
-    <cfRule type="expression" dxfId="27" priority="20">
-      <formula>U7&lt;U6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V7">
-    <cfRule type="expression" dxfId="26" priority="25">
-      <formula>V7&lt;V6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V13:X14 C15:E17">
-    <cfRule type="expression" dxfId="25" priority="47">
-      <formula>C13&lt;C12</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V15:Z17">
-    <cfRule type="expression" dxfId="24" priority="46">
-      <formula>V15&lt;V14</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W8:W12">
-    <cfRule type="expression" dxfId="23" priority="35">
-      <formula>W8&lt;W7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y7:Z14">
-    <cfRule type="expression" dxfId="22" priority="26">
-      <formula>Y7&lt;Y6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA12">
-    <cfRule type="expression" dxfId="21" priority="19">
-      <formula>AA7&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA17">
-    <cfRule type="expression" dxfId="20" priority="24">
-      <formula>AA7&lt;AA6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC7">
-    <cfRule type="expression" dxfId="19" priority="21">
-      <formula>AC7&lt;AC6</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AI7 X7:X12 AD8:AD10">
-    <cfRule type="expression" dxfId="18" priority="27">
-      <formula>X7&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ12:AJ17">
-    <cfRule type="expression" dxfId="17" priority="31">
-      <formula>AJ12&lt;AJ11</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:D6">
-    <cfRule type="expression" dxfId="16" priority="16">
-      <formula>C6&lt;C5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6">
-    <cfRule type="expression" dxfId="15" priority="14">
-      <formula>B6&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F6">
-    <cfRule type="expression" dxfId="14" priority="4">
-      <formula>F6&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6">
-    <cfRule type="expression" dxfId="13" priority="2">
-      <formula>G6&lt;G5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6:J6 L6:O6">
-    <cfRule type="expression" dxfId="12" priority="11">
-      <formula>G6&lt;G5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P6 S6 X6:Y6">
-    <cfRule type="expression" dxfId="11" priority="13">
-      <formula>P6&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K6">
-    <cfRule type="expression" dxfId="10" priority="6">
-      <formula>K6&lt;K5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q6">
-    <cfRule type="expression" dxfId="9" priority="17">
-      <formula>Q6&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R6">
-    <cfRule type="expression" dxfId="8" priority="15">
-      <formula>R6&lt;R5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6">
-    <cfRule type="expression" dxfId="7" priority="5">
-      <formula>E6&lt;E5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC6">
-    <cfRule type="expression" dxfId="6" priority="10">
-      <formula>AC6&lt;AC5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA6">
-    <cfRule type="expression" dxfId="5" priority="1">
-      <formula>AA6&lt;AA5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA6">
-    <cfRule type="expression" dxfId="4" priority="8">
-      <formula>AA6&lt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD6">
-    <cfRule type="expression" dxfId="3" priority="7">
-      <formula>AD6&lt;AD5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U6">
-    <cfRule type="expression" dxfId="2" priority="9">
-      <formula>U6&lt;U5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ6:AJ11">
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>AJ6&lt;AJ5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T6:W6 Z6 AB6 AE6:AI6">
-    <cfRule type="expression" dxfId="0" priority="12">
-      <formula>T6&lt;T5</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.1" right="0.5" top="0.32" bottom="0.25" header="0.25" footer="0.25"/>
@@ -17072,8 +16661,8 @@
       </c>
       <c r="B3" s="468"/>
       <c r="C3" s="468"/>
-      <c r="K3" s="896"/>
-      <c r="L3" s="896"/>
+      <c r="K3" s="898"/>
+      <c r="L3" s="898"/>
       <c r="M3" s="498"/>
       <c r="AH3" s="291"/>
       <c r="AI3" s="291"/>
@@ -17219,7 +16808,7 @@
         <v>31</v>
       </c>
       <c r="AG6" s="291"/>
-      <c r="AI6" s="895" t="s">
+      <c r="AI6" s="897" t="s">
         <v>216</v>
       </c>
     </row>
@@ -17324,7 +16913,7 @@
       <c r="AH7" s="477" t="s">
         <v>19</v>
       </c>
-      <c r="AI7" s="895"/>
+      <c r="AI7" s="897"/>
       <c r="AJ7" s="292" t="s">
         <v>229</v>
       </c>
@@ -17831,8 +17420,12 @@
       <c r="I12" s="494">
         <v>345.5</v>
       </c>
-      <c r="J12" s="494"/>
-      <c r="K12" s="494"/>
+      <c r="J12" s="494">
+        <v>343.9</v>
+      </c>
+      <c r="K12" s="494">
+        <v>415.9</v>
+      </c>
       <c r="L12" s="494"/>
       <c r="M12" s="494"/>
       <c r="N12" s="494"/>
@@ -17856,7 +17449,7 @@
       <c r="AG12" s="494"/>
       <c r="AH12" s="495">
         <f>SUM(B12:AF12)</f>
-        <v>1936.2</v>
+        <v>2696</v>
       </c>
       <c r="AI12" s="496"/>
       <c r="AJ12" s="469"/>
@@ -17888,8 +17481,12 @@
       <c r="I13" s="682" t="s">
         <v>312</v>
       </c>
-      <c r="J13" s="669"/>
-      <c r="K13" s="669"/>
+      <c r="J13" s="669" t="s">
+        <v>307</v>
+      </c>
+      <c r="K13" s="1026" t="s">
+        <v>313</v>
+      </c>
       <c r="L13" s="669"/>
       <c r="M13" s="798"/>
       <c r="N13" s="798"/>
@@ -17948,8 +17545,12 @@
         <f>2+5</f>
         <v>7</v>
       </c>
-      <c r="J14" s="498"/>
-      <c r="K14" s="498"/>
+      <c r="J14" s="498">
+        <v>7</v>
+      </c>
+      <c r="K14" s="498">
+        <v>8</v>
+      </c>
       <c r="L14" s="498"/>
       <c r="M14" s="498"/>
       <c r="N14" s="498"/>
@@ -17973,7 +17574,7 @@
       <c r="AG14" s="498"/>
       <c r="AH14" s="468">
         <f>SUM(B14:AF14)</f>
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:149" s="504" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -18014,7 +17615,7 @@
       <c r="AG15" s="718"/>
       <c r="AH15" s="500">
         <f>IF(AH12=0,"",+(AH36*10)/AH12)</f>
-        <v>7.6696622249767588</v>
+        <v>5.508160237388724</v>
       </c>
       <c r="AI15" s="502"/>
       <c r="AJ15" s="503"/>
@@ -25124,34 +24725,39 @@
         <v>1600</v>
       </c>
       <c r="C74" s="888">
-        <v>1142</v>
-      </c>
-      <c r="D74" s="877">
-        <v>0</v>
-      </c>
-      <c r="E74" s="877">
-        <v>0</v>
-      </c>
-      <c r="F74" s="790">
-        <v>1583</v>
-      </c>
-      <c r="G74" s="790">
-        <v>1504</v>
-      </c>
-      <c r="H74" s="790">
-        <v>1416</v>
-      </c>
-      <c r="I74" s="790">
-        <v>1772</v>
-      </c>
-      <c r="J74" s="791">
-        <v>1532</v>
+        <v>1200</v>
+      </c>
+      <c r="D74" s="895">
+        <v>0</v>
+      </c>
+      <c r="E74" s="895">
+        <v>0</v>
+      </c>
+      <c r="F74" s="895">
+        <v>1600</v>
+      </c>
+      <c r="G74" s="895">
+        <v>1500</v>
+      </c>
+      <c r="H74" s="895">
+        <v>1400</v>
+      </c>
+      <c r="I74" s="896">
+        <f>2200+800</f>
+        <v>3000</v>
+      </c>
+      <c r="J74" s="877">
+        <v>1700</v>
       </c>
       <c r="K74" s="877">
-        <v>361</v>
-      </c>
-      <c r="L74" s="877"/>
-      <c r="M74" s="877"/>
+        <v>800</v>
+      </c>
+      <c r="L74" s="877">
+        <v>0</v>
+      </c>
+      <c r="M74" s="877">
+        <v>0</v>
+      </c>
       <c r="N74" s="877"/>
       <c r="O74" s="877"/>
       <c r="P74" s="877"/>
@@ -25174,7 +24780,7 @@
       <c r="AG74" s="790"/>
       <c r="AH74" s="516">
         <f>SUM(B74:AF74)</f>
-        <v>10910</v>
+        <v>12800</v>
       </c>
       <c r="AI74" s="537"/>
       <c r="AJ74" s="537"/>
@@ -27028,7 +26634,7 @@
       </c>
       <c r="C92" s="653">
         <f t="shared" si="35"/>
-        <v>4.0277072399977429</v>
+        <v>4.232266802099204</v>
       </c>
       <c r="D92" s="653" t="str">
         <f t="shared" si="35"/>
@@ -27040,23 +26646,23 @@
       </c>
       <c r="F92" s="653">
         <f t="shared" si="35"/>
-        <v>4.8483623377498448</v>
+        <v>4.9004294001261863</v>
       </c>
       <c r="G92" s="653">
         <f>IF(G$9=0,"",+G74/G$9)</f>
-        <v>4.2106206186028805</v>
+        <v>4.199422159510851</v>
       </c>
       <c r="H92" s="653">
         <f>IF(H$9=0,"",+H74/H$9)</f>
-        <v>3.4840119283120257</v>
+        <v>3.4446445618904211</v>
       </c>
       <c r="I92" s="653">
         <f t="shared" si="35"/>
-        <v>4.9056248581189195</v>
+        <v>8.3052339584406081</v>
       </c>
       <c r="J92" s="653">
         <f t="shared" si="35"/>
-        <v>4.9662219110229371</v>
+        <v>5.5108206584458186</v>
       </c>
       <c r="K92" s="653" t="str">
         <f t="shared" si="35"/>
@@ -27149,18 +26755,18 @@
       <c r="AG92" s="628"/>
       <c r="AH92" s="670">
         <f>IF(AH$9=0,"0",+(AH74)/AH$9)</f>
-        <v>4.5252344660439023</v>
+        <v>5.3091660096573738</v>
       </c>
       <c r="AI92" s="674">
         <v>5</v>
       </c>
       <c r="AJ92" s="675">
         <f>AI92-AH92</f>
-        <v>0.47476553395609766</v>
+        <v>-0.30916600965737384</v>
       </c>
       <c r="AK92" s="673">
         <f t="shared" si="34"/>
-        <v>90.504689320878057</v>
+        <v>106.18332019314747</v>
       </c>
       <c r="AL92" s="629"/>
       <c r="AM92" s="630"/>
@@ -29000,45 +28606,45 @@
   </mergeCells>
   <phoneticPr fontId="32" type="noConversion"/>
   <conditionalFormatting sqref="B93:C93 AH93">
-    <cfRule type="cellIs" dxfId="82" priority="127" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="127" operator="greaterThan">
       <formula>$AI$93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B90:AF90">
-    <cfRule type="cellIs" dxfId="81" priority="36" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="34" priority="36" operator="greaterThan">
       <formula>10.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92:AF92">
-    <cfRule type="cellIs" dxfId="80" priority="26" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="26" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="27" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="32" priority="27" operator="lessThanOrEqual">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93:AF93">
-    <cfRule type="cellIs" dxfId="78" priority="34" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="34" operator="greaterThan">
       <formula>1.7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94:AF94">
-    <cfRule type="cellIs" dxfId="77" priority="33" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="33" operator="greaterThan">
       <formula>22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:AF96">
-    <cfRule type="cellIs" dxfId="76" priority="32" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="32" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:AG22">
-    <cfRule type="cellIs" dxfId="75" priority="101" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="28" priority="101" operator="greaterThan">
       <formula>400</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42:AG42">
-    <cfRule type="cellIs" dxfId="74" priority="47" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="47" operator="greaterThan">
       <formula>70</formula>
     </cfRule>
   </conditionalFormatting>
@@ -29053,129 +28659,129 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94:AG94">
-    <cfRule type="cellIs" dxfId="73" priority="1174" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1174" operator="greaterThan">
       <formula>$AI$94</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:AG96">
-    <cfRule type="cellIs" dxfId="72" priority="1176" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="25" priority="1176" operator="greaterThan">
       <formula>$AI$96</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:AH15">
-    <cfRule type="cellIs" dxfId="71" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="1" operator="greaterThan">
       <formula>3.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B54:AH54">
-    <cfRule type="cellIs" dxfId="70" priority="123" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="123" operator="greaterThan">
       <formula>3.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B56:AH56">
-    <cfRule type="cellIs" dxfId="69" priority="61" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="22" priority="61" operator="greaterThan">
       <formula>0.1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B57:AH57 B59:AH59 B61:AH61">
-    <cfRule type="cellIs" dxfId="68" priority="62" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="62" operator="greaterThan">
       <formula>0.7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58:AH58 B62:AH62">
-    <cfRule type="cellIs" dxfId="67" priority="63" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="63" operator="greaterThan">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B60:AH60">
-    <cfRule type="cellIs" dxfId="66" priority="22" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="19" priority="22" operator="greaterThan">
       <formula>2.1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B65:AH65">
-    <cfRule type="cellIs" dxfId="65" priority="56" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="56" operator="greaterThan">
       <formula>0.3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68:AH68">
-    <cfRule type="cellIs" dxfId="64" priority="58" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="58" operator="greaterThan">
       <formula>9.6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:AH69">
-    <cfRule type="cellIs" dxfId="63" priority="59" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="59" operator="greaterThan">
       <formula>2.9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92:AH92">
-    <cfRule type="cellIs" dxfId="62" priority="48" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="48" operator="greaterThan">
       <formula>5.04</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93:AH93">
-    <cfRule type="cellIs" dxfId="61" priority="44" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="44" operator="greaterThan">
       <formula>1.7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="43" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="43" operator="greaterThan">
       <formula>1.7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:AH96">
-    <cfRule type="cellIs" dxfId="59" priority="37" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="37" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E96">
-    <cfRule type="cellIs" dxfId="58" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="39" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I63:AH63">
-    <cfRule type="cellIs" dxfId="57" priority="68" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="68" operator="greaterThan">
       <formula>0.6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC54:AG54">
-    <cfRule type="cellIs" dxfId="56" priority="82" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="82" operator="greaterThan">
       <formula>$AI$54</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC55:AG59 AC61:AG61 AC63:AG63 B64:AG64">
-    <cfRule type="cellIs" dxfId="55" priority="1135" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1135" operator="greaterThan">
       <formula>$AI59</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH94">
-    <cfRule type="cellIs" dxfId="54" priority="28" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="7" priority="28" operator="lessThanOrEqual">
       <formula>22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH94:AH96 B90:AH90 AH91">
-    <cfRule type="cellIs" dxfId="53" priority="1168" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="1168" operator="greaterThan">
       <formula>$AI$90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH96">
-    <cfRule type="cellIs" dxfId="52" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="29" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="30" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="30" operator="lessThan">
       <formula>7.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="40" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="40" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ8">
-    <cfRule type="cellIs" dxfId="49" priority="105" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="105" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="106" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="106" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK90:AK96">
-    <cfRule type="cellIs" dxfId="47" priority="50" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="50" operator="greaterThan">
       <formula>100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -31478,24 +31084,24 @@
     </row>
     <row r="6" spans="1:20" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="924" t="s">
+      <c r="A7" s="926" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="383"/>
       <c r="C7" s="383"/>
-      <c r="D7" s="937" t="s">
+      <c r="D7" s="939" t="s">
         <v>254</v>
       </c>
-      <c r="E7" s="940" t="s">
+      <c r="E7" s="942" t="s">
         <v>286</v>
       </c>
-      <c r="F7" s="934" t="s">
+      <c r="F7" s="936" t="s">
         <v>287</v>
       </c>
-      <c r="G7" s="930" t="s">
+      <c r="G7" s="932" t="s">
         <v>255</v>
       </c>
-      <c r="H7" s="930" t="s">
+      <c r="H7" s="932" t="s">
         <v>256</v>
       </c>
       <c r="I7" s="383" t="s">
@@ -31507,33 +31113,33 @@
       <c r="K7" s="390" t="s">
         <v>53</v>
       </c>
-      <c r="L7" s="931" t="s">
+      <c r="L7" s="933" t="s">
         <v>17</v>
       </c>
-      <c r="M7" s="932"/>
-      <c r="N7" s="932"/>
-      <c r="O7" s="932"/>
-      <c r="P7" s="933"/>
-      <c r="Q7" s="928" t="s">
+      <c r="M7" s="934"/>
+      <c r="N7" s="934"/>
+      <c r="O7" s="934"/>
+      <c r="P7" s="935"/>
+      <c r="Q7" s="930" t="s">
         <v>11</v>
       </c>
-      <c r="R7" s="929"/>
-      <c r="S7" s="929"/>
-      <c r="T7" s="929"/>
+      <c r="R7" s="931"/>
+      <c r="S7" s="931"/>
+      <c r="T7" s="931"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8" s="925"/>
+      <c r="A8" s="927"/>
       <c r="B8" s="384" t="s">
         <v>257</v>
       </c>
       <c r="C8" s="384" t="s">
         <v>258</v>
       </c>
-      <c r="D8" s="938"/>
-      <c r="E8" s="941"/>
-      <c r="F8" s="935"/>
-      <c r="G8" s="930"/>
-      <c r="H8" s="930"/>
+      <c r="D8" s="940"/>
+      <c r="E8" s="943"/>
+      <c r="F8" s="937"/>
+      <c r="G8" s="932"/>
+      <c r="H8" s="932"/>
       <c r="I8" s="383"/>
       <c r="J8" s="383"/>
       <c r="K8" s="390"/>
@@ -31556,12 +31162,12 @@
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="926"/>
+      <c r="A9" s="928"/>
       <c r="B9" s="385"/>
       <c r="C9" s="385"/>
-      <c r="D9" s="939"/>
-      <c r="E9" s="942"/>
-      <c r="F9" s="936"/>
+      <c r="D9" s="941"/>
+      <c r="E9" s="944"/>
+      <c r="F9" s="938"/>
       <c r="G9" s="383" t="s">
         <v>56</v>
       </c>
@@ -31726,7 +31332,7 @@
       </c>
       <c r="K11" s="722">
         <f>'CO2'!E8</f>
-        <v>1142</v>
+        <v>1200</v>
       </c>
       <c r="L11" s="723">
         <f>+'PROD.FIG. '!F6</f>
@@ -31963,7 +31569,7 @@
       </c>
       <c r="K14" s="722">
         <f>'CO2'!E11</f>
-        <v>1583</v>
+        <v>1600</v>
       </c>
       <c r="L14" s="723">
         <f>+'PROD.FIG. '!F9</f>
@@ -32042,7 +31648,7 @@
       </c>
       <c r="K15" s="722">
         <f>'CO2'!E12</f>
-        <v>1504</v>
+        <v>1500</v>
       </c>
       <c r="L15" s="723">
         <f>+'PROD.FIG. '!F10</f>
@@ -32121,7 +31727,7 @@
       </c>
       <c r="K16" s="722">
         <f>'CO2'!E13</f>
-        <v>1416</v>
+        <v>1400</v>
       </c>
       <c r="L16" s="723">
         <f>+'PROD.FIG. '!F11</f>
@@ -32200,7 +31806,7 @@
       </c>
       <c r="K17" s="722">
         <f>'CO2'!E14</f>
-        <v>1772</v>
+        <v>3000</v>
       </c>
       <c r="L17" s="723">
         <f>+'PROD.FIG. '!F12</f>
@@ -32279,7 +31885,7 @@
       </c>
       <c r="K18" s="722">
         <f>'CO2'!E15</f>
-        <v>1532</v>
+        <v>1700</v>
       </c>
       <c r="L18" s="723">
         <f>+'PROD.FIG. '!F13</f>
@@ -32358,7 +31964,7 @@
       </c>
       <c r="K19" s="775">
         <f>'CO2'!E16</f>
-        <v>361</v>
+        <v>800</v>
       </c>
       <c r="L19" s="776">
         <f>+'PROD.FIG. '!F14</f>
@@ -34124,7 +33730,7 @@
       </c>
       <c r="K43" s="20">
         <f t="shared" si="7"/>
-        <v>10910</v>
+        <v>12800</v>
       </c>
       <c r="L43" s="20">
         <f t="shared" si="7"/>
@@ -34199,7 +33805,7 @@
       </c>
       <c r="T44" s="399">
         <f>IF(S44=0,0,K43/P43)</f>
-        <v>4.5252344660439023</v>
+        <v>5.3091660096573738</v>
       </c>
     </row>
     <row r="45" spans="1:32" ht="15" x14ac:dyDescent="0.2">
@@ -34232,12 +33838,12 @@
       <c r="T46" s="2"/>
     </row>
     <row r="47" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="D47" s="927"/>
-      <c r="E47" s="927"/>
-      <c r="F47" s="927"/>
-      <c r="G47" s="927"/>
-      <c r="H47" s="927"/>
-      <c r="I47" s="927"/>
+      <c r="D47" s="929"/>
+      <c r="E47" s="929"/>
+      <c r="F47" s="929"/>
+      <c r="G47" s="929"/>
+      <c r="H47" s="929"/>
+      <c r="I47" s="929"/>
       <c r="AF47" t="s">
         <v>55</v>
       </c>
@@ -34276,41 +33882,41 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="Q10:Q44">
-    <cfRule type="cellIs" dxfId="109" priority="7" operator="between">
+    <cfRule type="cellIs" dxfId="62" priority="7" operator="between">
       <formula>0</formula>
       <formula>22</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="61" priority="8" operator="greaterThan">
       <formula>22</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="60" priority="9" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R10:R44">
-    <cfRule type="cellIs" dxfId="106" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="59" priority="1" operator="between">
       <formula>0</formula>
       <formula>10.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="58" priority="2" operator="greaterThan">
       <formula>10.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S10:S44">
-    <cfRule type="cellIs" dxfId="104" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="57" priority="3" operator="between">
       <formula>0</formula>
       <formula>7.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="56" priority="4" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T10:T44">
-    <cfRule type="cellIs" dxfId="102" priority="5" operator="between">
+    <cfRule type="cellIs" dxfId="55" priority="5" operator="between">
       <formula>0</formula>
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="54" priority="6" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -34342,16 +33948,16 @@
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="943" t="s">
+      <c r="A3" s="945" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="945" t="s">
+      <c r="B3" s="947" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="944"/>
-      <c r="B4" s="946"/>
+      <c r="A4" s="946"/>
+      <c r="B4" s="948"/>
     </row>
     <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="36">
@@ -34715,31 +34321,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="955" t="s">
+      <c r="A1" s="957" t="s">
         <v>304</v>
       </c>
-      <c r="B1" s="956"/>
-      <c r="C1" s="956"/>
-      <c r="D1" s="956"/>
-      <c r="E1" s="956"/>
-      <c r="F1" s="956"/>
-      <c r="G1" s="956"/>
-      <c r="H1" s="956"/>
-      <c r="I1" s="956"/>
-      <c r="J1" s="956"/>
-      <c r="K1" s="956"/>
-      <c r="L1" s="956"/>
-      <c r="M1" s="956"/>
+      <c r="B1" s="958"/>
+      <c r="C1" s="958"/>
+      <c r="D1" s="958"/>
+      <c r="E1" s="958"/>
+      <c r="F1" s="958"/>
+      <c r="G1" s="958"/>
+      <c r="H1" s="958"/>
+      <c r="I1" s="958"/>
+      <c r="J1" s="958"/>
+      <c r="K1" s="958"/>
+      <c r="L1" s="958"/>
+      <c r="M1" s="958"/>
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
       <c r="F2" s="9"/>
-      <c r="M2" s="947" t="s">
+      <c r="M2" s="949" t="s">
         <v>296</v>
       </c>
-      <c r="N2" s="947" t="s">
+      <c r="N2" s="949" t="s">
         <v>297</v>
       </c>
     </row>
@@ -34748,11 +34354,11 @@
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="9"/>
-      <c r="M3" s="948"/>
-      <c r="N3" s="948"/>
+      <c r="M3" s="950"/>
+      <c r="N3" s="950"/>
     </row>
     <row r="4" spans="1:17" s="339" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="961" t="s">
+      <c r="A4" s="963" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="847" t="s">
@@ -34785,22 +34391,22 @@
       <c r="K4" s="848" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="957" t="s">
+      <c r="L4" s="959" t="s">
         <v>243</v>
       </c>
-      <c r="M4" s="959" t="s">
+      <c r="M4" s="961" t="s">
         <v>246</v>
       </c>
-      <c r="N4" s="949" t="s">
+      <c r="N4" s="951" t="s">
         <v>246</v>
       </c>
-      <c r="O4" s="952" t="s">
+      <c r="O4" s="954" t="s">
         <v>298</v>
       </c>
       <c r="P4" s="350"/>
     </row>
     <row r="5" spans="1:17" s="339" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="962"/>
+      <c r="A5" s="964"/>
       <c r="B5" s="864" t="s">
         <v>41</v>
       </c>
@@ -34831,10 +34437,10 @@
       <c r="K5" s="865" t="s">
         <v>44</v>
       </c>
-      <c r="L5" s="958"/>
-      <c r="M5" s="960"/>
-      <c r="N5" s="950"/>
-      <c r="O5" s="953"/>
+      <c r="L5" s="960"/>
+      <c r="M5" s="962"/>
+      <c r="N5" s="952"/>
+      <c r="O5" s="955"/>
       <c r="P5" s="350"/>
     </row>
     <row r="6" spans="1:17" s="73" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -34851,8 +34457,8 @@
       <c r="K6" s="836"/>
       <c r="L6" s="869"/>
       <c r="M6" s="833"/>
-      <c r="N6" s="951"/>
-      <c r="O6" s="954"/>
+      <c r="N6" s="953"/>
+      <c r="O6" s="956"/>
       <c r="P6" s="350"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -37242,27 +36848,27 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="C7:C37">
-    <cfRule type="cellIs" dxfId="100" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="13" operator="greaterThan">
       <formula>24</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M7:N37">
-    <cfRule type="cellIs" dxfId="99" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="52" priority="9" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="11" operator="between">
+    <cfRule type="cellIs" dxfId="51" priority="11" operator="between">
       <formula>0</formula>
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M7:N38">
-    <cfRule type="cellIs" dxfId="97" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="lessThan">
       <formula>7.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="4" operator="greaterThan">
       <formula>7.2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -37306,120 +36912,120 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="955"/>
-      <c r="B1" s="956"/>
-      <c r="C1" s="956"/>
-      <c r="D1" s="956"/>
-      <c r="E1" s="956"/>
-      <c r="F1" s="956"/>
-      <c r="G1" s="956"/>
-      <c r="H1" s="956"/>
-      <c r="I1" s="956"/>
-      <c r="J1" s="956"/>
-      <c r="K1" s="956"/>
-      <c r="L1" s="956"/>
-      <c r="M1" s="956"/>
-      <c r="N1" s="956"/>
-      <c r="O1" s="956"/>
-      <c r="P1" s="956"/>
-      <c r="Q1" s="956"/>
-      <c r="R1" s="956"/>
-      <c r="S1" s="956"/>
-      <c r="T1" s="956"/>
-      <c r="U1" s="956"/>
-      <c r="V1" s="956"/>
-      <c r="W1" s="956"/>
-      <c r="X1" s="956"/>
-      <c r="Y1" s="956"/>
-      <c r="Z1" s="956"/>
-      <c r="AA1" s="956"/>
+      <c r="A1" s="957"/>
+      <c r="B1" s="958"/>
+      <c r="C1" s="958"/>
+      <c r="D1" s="958"/>
+      <c r="E1" s="958"/>
+      <c r="F1" s="958"/>
+      <c r="G1" s="958"/>
+      <c r="H1" s="958"/>
+      <c r="I1" s="958"/>
+      <c r="J1" s="958"/>
+      <c r="K1" s="958"/>
+      <c r="L1" s="958"/>
+      <c r="M1" s="958"/>
+      <c r="N1" s="958"/>
+      <c r="O1" s="958"/>
+      <c r="P1" s="958"/>
+      <c r="Q1" s="958"/>
+      <c r="R1" s="958"/>
+      <c r="S1" s="958"/>
+      <c r="T1" s="958"/>
+      <c r="U1" s="958"/>
+      <c r="V1" s="958"/>
+      <c r="W1" s="958"/>
+      <c r="X1" s="958"/>
+      <c r="Y1" s="958"/>
+      <c r="Z1" s="958"/>
+      <c r="AA1" s="958"/>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:31" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="967" t="s">
+      <c r="B4" s="969" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="965" t="s">
+      <c r="C4" s="967" t="s">
         <v>105</v>
       </c>
-      <c r="D4" s="963" t="s">
+      <c r="D4" s="965" t="s">
         <v>106</v>
       </c>
-      <c r="E4" s="965" t="s">
+      <c r="E4" s="967" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="963" t="s">
+      <c r="F4" s="965" t="s">
         <v>239</v>
       </c>
-      <c r="G4" s="963" t="s">
+      <c r="G4" s="965" t="s">
         <v>108</v>
       </c>
-      <c r="H4" s="963" t="s">
+      <c r="H4" s="965" t="s">
         <v>161</v>
       </c>
-      <c r="I4" s="965" t="s">
+      <c r="I4" s="967" t="s">
         <v>207</v>
       </c>
-      <c r="J4" s="965" t="s">
+      <c r="J4" s="967" t="s">
         <v>109</v>
       </c>
-      <c r="K4" s="965" t="s">
+      <c r="K4" s="967" t="s">
         <v>174</v>
       </c>
-      <c r="L4" s="965" t="s">
+      <c r="L4" s="967" t="s">
         <v>173</v>
       </c>
-      <c r="M4" s="965" t="s">
+      <c r="M4" s="967" t="s">
         <v>103</v>
       </c>
       <c r="N4" s="48"/>
       <c r="O4" s="48"/>
       <c r="P4" s="48"/>
       <c r="Q4" s="48"/>
-      <c r="R4" s="963" t="s">
+      <c r="R4" s="965" t="s">
         <v>110</v>
       </c>
-      <c r="S4" s="963" t="s">
+      <c r="S4" s="965" t="s">
         <v>240</v>
       </c>
       <c r="T4" s="48"/>
-      <c r="U4" s="965" t="s">
+      <c r="U4" s="967" t="s">
         <v>153</v>
       </c>
       <c r="V4" s="48"/>
       <c r="W4" s="48"/>
-      <c r="X4" s="965" t="s">
+      <c r="X4" s="967" t="s">
         <v>175</v>
       </c>
-      <c r="Y4" s="965" t="s">
+      <c r="Y4" s="967" t="s">
         <v>176</v>
       </c>
-      <c r="Z4" s="972" t="s">
+      <c r="Z4" s="974" t="s">
         <v>247</v>
       </c>
-      <c r="AA4" s="974" t="s">
+      <c r="AA4" s="976" t="s">
         <v>243</v>
       </c>
-      <c r="AB4" s="970" t="s">
+      <c r="AB4" s="972" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:31" s="300" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="968"/>
-      <c r="C5" s="966"/>
-      <c r="D5" s="964"/>
-      <c r="E5" s="969"/>
-      <c r="F5" s="964"/>
-      <c r="G5" s="964"/>
-      <c r="H5" s="964"/>
-      <c r="I5" s="969"/>
-      <c r="J5" s="969"/>
-      <c r="K5" s="969"/>
-      <c r="L5" s="969"/>
-      <c r="M5" s="969"/>
+      <c r="B5" s="970"/>
+      <c r="C5" s="968"/>
+      <c r="D5" s="966"/>
+      <c r="E5" s="971"/>
+      <c r="F5" s="966"/>
+      <c r="G5" s="966"/>
+      <c r="H5" s="966"/>
+      <c r="I5" s="971"/>
+      <c r="J5" s="971"/>
+      <c r="K5" s="971"/>
+      <c r="L5" s="971"/>
+      <c r="M5" s="971"/>
       <c r="N5" s="50" t="s">
         <v>111</v>
       </c>
@@ -37432,23 +37038,23 @@
       <c r="Q5" s="50" t="s">
         <v>113</v>
       </c>
-      <c r="R5" s="964"/>
-      <c r="S5" s="964"/>
+      <c r="R5" s="966"/>
+      <c r="S5" s="966"/>
       <c r="T5" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="U5" s="976"/>
+      <c r="U5" s="978"/>
       <c r="V5" s="80" t="s">
         <v>156</v>
       </c>
       <c r="W5" s="80" t="s">
         <v>157</v>
       </c>
-      <c r="X5" s="969"/>
-      <c r="Y5" s="969"/>
-      <c r="Z5" s="973"/>
-      <c r="AA5" s="975"/>
-      <c r="AB5" s="971"/>
+      <c r="X5" s="971"/>
+      <c r="Y5" s="971"/>
+      <c r="Z5" s="975"/>
+      <c r="AA5" s="977"/>
+      <c r="AB5" s="973"/>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B6" s="21" t="s">
@@ -41556,10 +41162,10 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="AB6:AB38">
-    <cfRule type="cellIs" dxfId="94" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="lessThan">
       <formula>10.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="greaterThan">
       <formula>10.2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41590,15 +41196,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="977" t="s">
+      <c r="A1" s="979" t="s">
         <v>303</v>
       </c>
-      <c r="B1" s="978"/>
-      <c r="C1" s="978"/>
-      <c r="D1" s="979"/>
-      <c r="E1" s="978"/>
-      <c r="F1" s="978"/>
-      <c r="G1" s="980"/>
+      <c r="B1" s="980"/>
+      <c r="C1" s="980"/>
+      <c r="D1" s="981"/>
+      <c r="E1" s="980"/>
+      <c r="F1" s="980"/>
+      <c r="G1" s="982"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B2" s="9"/>
@@ -41611,7 +41217,7 @@
       <c r="D3" s="359"/>
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="991" t="s">
+      <c r="A4" s="993" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="39" t="s">
@@ -41623,19 +41229,19 @@
       <c r="D4" s="361" t="s">
         <v>285</v>
       </c>
-      <c r="E4" s="981" t="s">
+      <c r="E4" s="983" t="s">
         <v>245</v>
       </c>
-      <c r="F4" s="984" t="s">
+      <c r="F4" s="986" t="s">
         <v>243</v>
       </c>
-      <c r="G4" s="987" t="s">
+      <c r="G4" s="989" t="s">
         <v>253</v>
       </c>
-      <c r="H4" s="990"/>
+      <c r="H4" s="992"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="992"/>
+      <c r="A5" s="994"/>
       <c r="B5" s="34" t="s">
         <v>48</v>
       </c>
@@ -41645,20 +41251,20 @@
       <c r="D5" s="361" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="982"/>
-      <c r="F5" s="985"/>
-      <c r="G5" s="988"/>
-      <c r="H5" s="990"/>
+      <c r="E5" s="984"/>
+      <c r="F5" s="987"/>
+      <c r="G5" s="990"/>
+      <c r="H5" s="992"/>
     </row>
     <row r="6" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="993"/>
+      <c r="A6" s="995"/>
       <c r="B6" s="40"/>
       <c r="C6" s="362"/>
       <c r="D6" s="361"/>
-      <c r="E6" s="983"/>
-      <c r="F6" s="986"/>
-      <c r="G6" s="989"/>
-      <c r="H6" s="990"/>
+      <c r="E6" s="985"/>
+      <c r="F6" s="988"/>
+      <c r="G6" s="991"/>
+      <c r="H6" s="992"/>
     </row>
     <row r="7" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A7" s="686">
@@ -42663,12 +42269,12 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="92" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="45" priority="1" operator="lessThan">
       <formula>22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G38">
-    <cfRule type="cellIs" dxfId="91" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="2" operator="greaterThan">
       <formula>21</formula>
     </cfRule>
   </conditionalFormatting>
@@ -42699,16 +42305,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="994" t="s">
+      <c r="A1" s="996" t="s">
         <v>302</v>
       </c>
-      <c r="B1" s="956"/>
-      <c r="C1" s="956"/>
-      <c r="D1" s="956"/>
-      <c r="E1" s="956"/>
-      <c r="F1" s="956"/>
-      <c r="G1" s="956"/>
-      <c r="H1" s="956"/>
+      <c r="B1" s="958"/>
+      <c r="C1" s="958"/>
+      <c r="D1" s="958"/>
+      <c r="E1" s="958"/>
+      <c r="F1" s="958"/>
+      <c r="G1" s="958"/>
+      <c r="H1" s="958"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D2" s="12"/>
@@ -43437,11 +43043,11 @@
       <c r="D3" s="85"/>
       <c r="E3" s="85"/>
       <c r="F3" s="1"/>
-      <c r="I3" s="999" t="s">
+      <c r="I3" s="1001" t="s">
         <v>267</v>
       </c>
-      <c r="J3" s="1000"/>
-      <c r="K3" s="1001"/>
+      <c r="J3" s="1002"/>
+      <c r="K3" s="1003"/>
     </row>
     <row r="4" spans="1:24" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
@@ -43454,46 +43060,46 @@
         <v>250</v>
       </c>
       <c r="H4" s="347"/>
-      <c r="I4" s="1002" t="s">
+      <c r="I4" s="1004" t="s">
         <v>262</v>
       </c>
-      <c r="J4" s="1003"/>
-      <c r="K4" s="1004"/>
+      <c r="J4" s="1005"/>
+      <c r="K4" s="1006"/>
       <c r="M4" s="417"/>
       <c r="N4" s="417"/>
       <c r="O4" s="418"/>
       <c r="P4" s="418"/>
-      <c r="Q4" s="1014" t="s">
+      <c r="Q4" s="1016" t="s">
         <v>283</v>
       </c>
-      <c r="R4" s="1014"/>
-      <c r="S4" s="1014"/>
-      <c r="T4" s="1014"/>
+      <c r="R4" s="1016"/>
+      <c r="S4" s="1016"/>
+      <c r="T4" s="1016"/>
       <c r="U4" s="191"/>
       <c r="V4" s="417"/>
       <c r="W4" s="191"/>
       <c r="X4" s="191"/>
     </row>
     <row r="5" spans="1:24" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="943" t="s">
+      <c r="A5" s="945" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="945" t="s">
+      <c r="B5" s="947" t="s">
         <v>251</v>
       </c>
-      <c r="C5" s="945" t="s">
+      <c r="C5" s="947" t="s">
         <v>282</v>
       </c>
-      <c r="D5" s="1021" t="s">
+      <c r="D5" s="1023" t="s">
         <v>279</v>
       </c>
-      <c r="E5" s="1021" t="s">
+      <c r="E5" s="1023" t="s">
         <v>280</v>
       </c>
-      <c r="F5" s="1019" t="s">
+      <c r="F5" s="1021" t="s">
         <v>243</v>
       </c>
-      <c r="G5" s="1016" t="s">
+      <c r="G5" s="1018" t="s">
         <v>249</v>
       </c>
       <c r="I5" s="419" t="s">
@@ -43505,43 +43111,43 @@
       <c r="K5" s="421" t="s">
         <v>265</v>
       </c>
-      <c r="M5" s="1005" t="s">
+      <c r="M5" s="1007" t="s">
         <v>266</v>
       </c>
-      <c r="N5" s="1006"/>
-      <c r="O5" s="1007"/>
+      <c r="N5" s="1008"/>
+      <c r="O5" s="1009"/>
       <c r="P5" s="422"/>
-      <c r="Q5" s="1008" t="s">
+      <c r="Q5" s="1010" t="s">
         <v>7</v>
       </c>
-      <c r="R5" s="1010" t="s">
+      <c r="R5" s="1012" t="s">
         <v>267</v>
       </c>
-      <c r="S5" s="1011"/>
+      <c r="S5" s="1013"/>
       <c r="T5" s="452" t="s">
         <v>268</v>
       </c>
       <c r="U5" s="423" t="s">
         <v>269</v>
       </c>
-      <c r="V5" s="1012" t="s">
+      <c r="V5" s="1014" t="s">
         <v>277</v>
       </c>
-      <c r="W5" s="995" t="s">
+      <c r="W5" s="997" t="s">
         <v>270</v>
       </c>
-      <c r="X5" s="997" t="s">
+      <c r="X5" s="999" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1015"/>
-      <c r="B6" s="1018"/>
-      <c r="C6" s="1018"/>
-      <c r="D6" s="1022"/>
-      <c r="E6" s="1022"/>
-      <c r="F6" s="1020"/>
-      <c r="G6" s="1017"/>
+      <c r="A6" s="1017"/>
+      <c r="B6" s="1020"/>
+      <c r="C6" s="1020"/>
+      <c r="D6" s="1024"/>
+      <c r="E6" s="1024"/>
+      <c r="F6" s="1022"/>
+      <c r="G6" s="1019"/>
       <c r="I6" s="424">
         <v>10</v>
       </c>
@@ -43560,7 +43166,7 @@
         <v>273</v>
       </c>
       <c r="P6" s="418"/>
-      <c r="Q6" s="1009"/>
+      <c r="Q6" s="1011"/>
       <c r="R6" s="448" t="s">
         <v>274</v>
       </c>
@@ -43573,9 +43179,9 @@
       <c r="U6" s="429" t="s">
         <v>275</v>
       </c>
-      <c r="V6" s="1013"/>
-      <c r="W6" s="996"/>
-      <c r="X6" s="998"/>
+      <c r="V6" s="1015"/>
+      <c r="W6" s="998"/>
+      <c r="X6" s="1000"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="715">
@@ -43678,14 +43284,14 @@
         <v>1141.6199999999953</v>
       </c>
       <c r="E8" s="716">
-        <v>1142</v>
+        <v>1200</v>
       </c>
       <c r="F8" s="717">
         <v>283.536</v>
       </c>
       <c r="G8" s="336">
         <f t="shared" ref="G8:G37" si="1">IF(F8=0,"0",(E8/F8))</f>
-        <v>4.0277072399977429</v>
+        <v>4.232266802099204</v>
       </c>
       <c r="I8" s="430">
         <v>30</v>
@@ -43905,14 +43511,14 @@
         <v>1583.3100000000559</v>
       </c>
       <c r="E11" s="768">
-        <v>1583</v>
+        <v>1600</v>
       </c>
       <c r="F11" s="769">
         <v>326.50200000000001</v>
       </c>
       <c r="G11" s="336">
         <f t="shared" si="1"/>
-        <v>4.8483623377498448</v>
+        <v>4.9004294001261863</v>
       </c>
       <c r="I11" s="430">
         <v>60</v>
@@ -43978,14 +43584,14 @@
         <v>1503.5599999999395</v>
       </c>
       <c r="E12" s="768">
-        <v>1504</v>
+        <v>1500</v>
       </c>
       <c r="F12" s="769">
         <v>357.19200000000001</v>
       </c>
       <c r="G12" s="336">
         <f>IF(F12=0,"0",(E12/F12))</f>
-        <v>4.2106206186028805</v>
+        <v>4.199422159510851</v>
       </c>
       <c r="I12" s="430">
         <v>70</v>
@@ -44051,14 +43657,14 @@
         <v>1416.1900000000605</v>
       </c>
       <c r="E13" s="716">
-        <v>1416</v>
+        <v>1400</v>
       </c>
       <c r="F13" s="717">
         <v>406.428</v>
       </c>
       <c r="G13" s="336">
         <f t="shared" si="1"/>
-        <v>3.4840119283120257</v>
+        <v>3.4446445618904211</v>
       </c>
       <c r="I13" s="430">
         <v>80</v>
@@ -44121,14 +43727,14 @@
         <v>1771.5</v>
       </c>
       <c r="E14" s="716">
-        <v>1772</v>
+        <v>3000</v>
       </c>
       <c r="F14" s="717">
         <v>361.21800000000002</v>
       </c>
       <c r="G14" s="336">
         <f t="shared" si="1"/>
-        <v>4.9056248581189195</v>
+        <v>8.3052339584406081</v>
       </c>
       <c r="I14" s="430">
         <v>90</v>
@@ -44194,14 +43800,14 @@
         <v>1532</v>
       </c>
       <c r="E15" s="716">
-        <v>1532</v>
+        <v>1700</v>
       </c>
       <c r="F15" s="717">
         <v>308.48400000000004</v>
       </c>
       <c r="G15" s="336">
         <f t="shared" si="1"/>
-        <v>4.9662219110229371</v>
+        <v>5.5108206584458186</v>
       </c>
       <c r="I15" s="430">
         <v>100</v>
@@ -44264,7 +43870,7 @@
         <v>360.76999999990221</v>
       </c>
       <c r="E16" s="716">
-        <v>361</v>
+        <v>800</v>
       </c>
       <c r="F16" s="717">
         <v>0</v>
@@ -45874,7 +45480,7 @@
       </c>
       <c r="E38" s="713">
         <f>SUM(E7:E37)</f>
-        <v>10910</v>
+        <v>12800</v>
       </c>
       <c r="F38" s="714">
         <f>SUM(F7:F37)</f>
@@ -45882,7 +45488,7 @@
       </c>
       <c r="G38" s="345">
         <f>IF(F38=0,"0",(E38/F38))</f>
-        <v>4.5252344660439023</v>
+        <v>5.3091660096573738</v>
       </c>
       <c r="H38" s="348">
         <v>5</v>
@@ -46063,10 +45669,10 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="G7:G38">
-    <cfRule type="cellIs" dxfId="90" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
       <formula>21</formula>
     </cfRule>
   </conditionalFormatting>
@@ -46360,7 +45966,7 @@
         <v>31</v>
       </c>
       <c r="AG6" s="293"/>
-      <c r="AH6" s="895" t="s">
+      <c r="AH6" s="897" t="s">
         <v>216</v>
       </c>
       <c r="AI6" s="291"/>
@@ -46465,7 +46071,7 @@
       <c r="AG7" s="212" t="s">
         <v>19</v>
       </c>
-      <c r="AH7" s="895"/>
+      <c r="AH7" s="897"/>
       <c r="AI7" s="292" t="s">
         <v>229</v>
       </c>
@@ -46830,11 +46436,11 @@
         <f>'Daily KPIs'!X10</f>
         <v>0</v>
       </c>
-      <c r="Y10" s="1023">
+      <c r="Y10" s="1025">
         <f>'Daily KPIs'!Y10</f>
         <v>0</v>
       </c>
-      <c r="Z10" s="1023"/>
+      <c r="Z10" s="1025"/>
       <c r="AA10" s="163">
         <f>'Daily KPIs'!AA10</f>
         <v>0</v>
@@ -51571,13 +51177,13 @@
         <f>IF(I$93=0,"",+(I28*10)/I$93)</f>
         <v>5.4124457308248912</v>
       </c>
-      <c r="J63" s="168" t="str">
+      <c r="J63" s="168">
         <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="K63" s="168" t="str">
+        <v>5.5830183192788603</v>
+      </c>
+      <c r="K63" s="168">
         <f t="shared" si="12"/>
-        <v/>
+        <v>3.8951671074777594</v>
       </c>
       <c r="L63" s="168" t="str">
         <f t="shared" si="12"/>
@@ -51665,14 +51271,14 @@
       </c>
       <c r="AG63" s="243">
         <f>IF(+(AG28*10)/AG$93&lt;1,0,+(AG28*10)/AG$93)</f>
-        <v>7.6696622249767588</v>
+        <v>5.508160237388724</v>
       </c>
       <c r="AH63" s="243">
         <v>2.5</v>
       </c>
       <c r="AI63" s="244">
         <f t="shared" si="11"/>
-        <v>-5.1696622249767588</v>
+        <v>-3.008160237388724</v>
       </c>
     </row>
     <row r="64" spans="1:37" s="90" customFormat="1" ht="18" x14ac:dyDescent="0.25">
@@ -53366,11 +52972,11 @@
       </c>
       <c r="J78" s="152">
         <f t="shared" si="37"/>
-        <v>11.345807237976683</v>
+        <v>16.928825557255546</v>
       </c>
       <c r="K78" s="152">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>3.8951671074777594</v>
       </c>
       <c r="L78" s="152">
         <f t="shared" si="37"/>
@@ -53458,7 +53064,7 @@
       </c>
       <c r="AG78" s="253">
         <f>SUM(AG62:AG77)</f>
-        <v>19.146585934915784</v>
+        <v>16.985083947327745</v>
       </c>
       <c r="AH78" s="253">
         <f t="shared" si="37"/>
@@ -53466,7 +53072,7 @@
       </c>
       <c r="AI78" s="253">
         <f t="shared" si="11"/>
-        <v>-3.546585934915786</v>
+        <v>-1.3850839473277468</v>
       </c>
       <c r="AJ78" s="210"/>
       <c r="AK78" s="210"/>
@@ -54968,11 +54574,11 @@
       </c>
       <c r="J93" s="165">
         <f>'Daily KPIs'!J12</f>
-        <v>0</v>
+        <v>343.9</v>
       </c>
       <c r="K93" s="165">
         <f>'Daily KPIs'!K12</f>
-        <v>0</v>
+        <v>415.9</v>
       </c>
       <c r="L93" s="165">
         <f>'Daily KPIs'!L12</f>
@@ -55060,7 +54666,7 @@
       </c>
       <c r="AG93" s="260">
         <f>SUM(B93:AF93)</f>
-        <v>1936.2</v>
+        <v>2696</v>
       </c>
       <c r="AH93" s="261"/>
       <c r="AI93" s="289"/>
@@ -55101,13 +54707,13 @@
         <f>'Daily KPIs'!I13</f>
         <v>ST/CB</v>
       </c>
-      <c r="J94" s="166">
+      <c r="J94" s="166" t="str">
         <f>'Daily KPIs'!J13</f>
-        <v>0</v>
-      </c>
-      <c r="K94" s="166">
+        <v>CB</v>
+      </c>
+      <c r="K94" s="166" t="str">
         <f>'Daily KPIs'!K13</f>
-        <v>0</v>
+        <v>GU</v>
       </c>
       <c r="L94" s="166">
         <f>'Daily KPIs'!L13</f>
@@ -55235,11 +54841,11 @@
       </c>
       <c r="J95" s="174">
         <f>'Daily KPIs'!J14</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K95" s="174">
         <f>'Daily KPIs'!K14</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L95" s="174">
         <f>'Daily KPIs'!L14</f>
@@ -55327,7 +54933,7 @@
       </c>
       <c r="AG95" s="262">
         <f>SUM($B95:AF95)</f>
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="AH95" s="262"/>
       <c r="AI95" s="290"/>
@@ -55891,30 +55497,30 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="B82:AF82">
-    <cfRule type="cellIs" dxfId="88" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="3" operator="greaterThan">
       <formula>26</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B84:AF84">
-    <cfRule type="cellIs" dxfId="87" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="40" priority="4" operator="greaterThan">
       <formula>6.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D64:D65 D67 T69:AI70 D71 D73:D77">
-    <cfRule type="cellIs" dxfId="86" priority="5" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="5" stopIfTrue="1" operator="greaterThan">
       <formula>3.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:S69 B70:S70">
-    <cfRule type="cellIs" dxfId="85" priority="13" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="13" stopIfTrue="1" operator="greaterThan">
       <formula>3.8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI8">
-    <cfRule type="cellIs" dxfId="84" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="37" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="36" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>